<commit_message>
RS485: on-board 120R terminator (R7) and 330R bias (R5/R9)
- R7 (between A and B) 10k -> 120R, R5/R9 470R -> 330R; '1' level 0.39 V with a second terminator
  at the far end (24/24 bits at 38400 baud), no external resistor needed
- BOM, JLCPCB BOM, Gerber, Excel purchase list and Order_Files regenerated

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Order_Files/Component_Order_List.xlsx
+++ b/Order_Files/Component_Order_List.xlsx
@@ -564,11 +564,11 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>R1,R2,R3,R6,R7,R11,R14,R18,R19,R20,R21,R22,R32,R35</t>
+          <t>R1,R2,R3,R6,R11,R14,R18,R19,R20,R21,R22,R32,R35</t>
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
@@ -581,10 +581,10 @@
         </is>
       </c>
       <c r="G2" s="2" t="n">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>0.6971000000000001</v>
+        <v>0.6969</v>
       </c>
       <c r="I2" s="4">
         <f>G2*H2</f>
@@ -647,20 +647,20 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Resistor 470R 0805 1%</t>
+          <t>Resistor 120R 0805 1%</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>R5,R9</t>
+          <t>R7</t>
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>0805W8F4700T5E</t>
+          <t>RC0805FR-07120RL</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -672,7 +672,7 @@
         <v>20</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>0.7565</v>
+        <v>0.731</v>
       </c>
       <c r="I4" s="4">
         <f>G4*H4</f>
@@ -685,7 +685,7 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>RS485 bias; min order 20</t>
+          <t>RS485 on-board terminator between A and B; min order 20</t>
         </is>
       </c>
     </row>
@@ -748,11 +748,11 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>R4,R10,R29,R30</t>
+          <t>R4,R5,R9,R10,R29,R30</t>
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
@@ -765,7 +765,7 @@
         </is>
       </c>
       <c r="G6" s="2" t="n">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="H6" s="4" t="n">
         <v>0.7309</v>
@@ -779,7 +779,11 @@
           <t>ex-GST (18% GST extra)</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr"/>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>R5,R9 = RS485 bias resistors</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">

</xml_diff>

<commit_message>
Purchase list: external 5V SMPS, so no AC mains parts (HLK-10M05, MOV, fuse, NTC, X2 cap, J1)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Order_Files/Component_Order_List.xlsx
+++ b/Order_Files/Component_Order_List.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K15"/>
+  <dimension ref="A1:K13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -800,12 +800,12 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Varistor MOV 14D471K</t>
+          <t>Female header 2x8 2.54mm</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>RV1</t>
+          <t>J3</t>
         </is>
       </c>
       <c r="D7" s="2" t="n">
@@ -813,7 +813,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>MOV-14D471K</t>
+          <t>2X8 16Pin Female Berg Strip</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
@@ -825,7 +825,7 @@
         <v>6</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>14.53</v>
+        <v>11.92</v>
       </c>
       <c r="I7" s="4">
         <f>G7*H7</f>
@@ -838,7 +838,7 @@
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>Mains input protection</t>
+          <t>P10 panel connector</t>
         </is>
       </c>
     </row>
@@ -848,12 +848,12 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Female header 2x8 2.54mm</t>
+          <t>Right-angle male header 7x1 2.54mm (use 6 pins)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>J3</t>
+          <t>J2</t>
         </is>
       </c>
       <c r="D8" s="2" t="n">
@@ -861,7 +861,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>2X8 16Pin Female Berg Strip</t>
+          <t>7x1 7Pin Male Right Angle</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
@@ -873,7 +873,7 @@
         <v>6</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>11.92</v>
+        <v>5.18</v>
       </c>
       <c r="I8" s="4">
         <f>G8*H8</f>
@@ -886,7 +886,7 @@
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>P10 panel connector</t>
+          <t>FTDI programming header</t>
         </is>
       </c>
     </row>
@@ -896,12 +896,12 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Right-angle male header 7x1 2.54mm (use 6 pins)</t>
+          <t>MOSFET P-ch SI2301</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>J2</t>
+          <t>Q3</t>
         </is>
       </c>
       <c r="D9" s="2" t="n">
@@ -909,7 +909,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>7x1 7Pin Male Right Angle</t>
+          <t>SI2301CDS-T1-GE3</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
@@ -921,7 +921,7 @@
         <v>6</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>5.18</v>
+        <v>24.69</v>
       </c>
       <c r="I9" s="4">
         <f>G9*H9</f>
@@ -934,7 +934,7 @@
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>FTDI programming header</t>
+          <t>5V DC input reverse-polarity protection</t>
         </is>
       </c>
     </row>
@@ -944,12 +944,12 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>MOSFET P-ch SI2301</t>
+          <t>LDO 3.3V SOT-223</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Q3</t>
+          <t>VR1</t>
         </is>
       </c>
       <c r="D10" s="2" t="n">
@@ -957,7 +957,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>SI2301CDS-T1-GE3</t>
+          <t>LM1117GS 3.3V</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
@@ -969,7 +969,7 @@
         <v>6</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>24.69</v>
+        <v>13.75</v>
       </c>
       <c r="I10" s="4">
         <f>G10*H10</f>
@@ -982,7 +982,7 @@
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>5V DC input reverse-polarity protection</t>
+          <t>Generic LM1117-3.3 instead of TI LM1117IMPX-3.3</t>
         </is>
       </c>
     </row>
@@ -992,20 +992,20 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>LDO 3.3V SOT-223</t>
+          <t>Transistor NPN SOT-23</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>VR1</t>
+          <t>Q1,Q2</t>
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>LM1117GS 3.3V</t>
+          <t>BC848 30V 100mA</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
@@ -1014,10 +1014,10 @@
         </is>
       </c>
       <c r="G11" s="2" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>13.75</v>
+        <v>3.46</v>
       </c>
       <c r="I11" s="4">
         <f>G11*H11</f>
@@ -1030,7 +1030,7 @@
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>Generic LM1117-3.3 instead of TI LM1117IMPX-3.3</t>
+          <t>Auto-reset / auto-boot (DTR, RTS)</t>
         </is>
       </c>
     </row>
@@ -1040,32 +1040,32 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Transistor NPN SOT-23</t>
+          <t>TVS diode 5V unidirectional</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Q1,Q2</t>
+          <t>D7</t>
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>BC848 30V 100mA</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>Sharvi Electronics</t>
+          <t>SMAJ5.0A (Littelfuse)</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>Robu.in</t>
         </is>
       </c>
       <c r="G12" s="2" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>3.46</v>
+        <v>21</v>
       </c>
       <c r="I12" s="4">
         <f>G12*H12</f>
@@ -1073,12 +1073,12 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>ex-GST (18% GST extra)</t>
+          <t>incl. GST</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>Auto-reset / auto-boot (DTR, RTS)</t>
+          <t>5V rail protection</t>
         </is>
       </c>
     </row>
@@ -1088,12 +1088,12 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>5V 10W AC-DC module</t>
+          <t>LED 0805 green (yellow-green 571nm)</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>PS1</t>
+          <t>D8</t>
         </is>
       </c>
       <c r="D13" s="2" t="n">
@@ -1101,7 +1101,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>HLK-10M05</t>
+          <t>LTST-C171KGKT (Lite-On)</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
@@ -1113,7 +1113,7 @@
         <v>6</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>322</v>
+        <v>2.46</v>
       </c>
       <c r="I13" s="4">
         <f>G13*H13</f>
@@ -1124,99 +1124,7 @@
           <t>incl. GST</t>
         </is>
       </c>
-      <c r="K13" s="2" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>TVS diode 5V unidirectional</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>D7</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>SMAJ5.0A (Littelfuse)</t>
-        </is>
-      </c>
-      <c r="F14" s="5" t="inlineStr">
-        <is>
-          <t>Robu.in</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="H14" s="4" t="n">
-        <v>21</v>
-      </c>
-      <c r="I14" s="4">
-        <f>G14*H14</f>
-        <v/>
-      </c>
-      <c r="J14" s="2" t="inlineStr">
-        <is>
-          <t>incl. GST</t>
-        </is>
-      </c>
-      <c r="K14" s="2" t="inlineStr">
-        <is>
-          <t>5V rail protection</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="n">
-        <v>14</v>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>LED 0805 green (yellow-green 571nm)</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>D8</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>LTST-C171KGKT (Lite-On)</t>
-        </is>
-      </c>
-      <c r="F15" s="5" t="inlineStr">
-        <is>
-          <t>Robu.in</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="H15" s="4" t="n">
-        <v>2.27</v>
-      </c>
-      <c r="I15" s="4">
-        <f>G15*H15</f>
-        <v/>
-      </c>
-      <c r="J15" s="2" t="inlineStr">
-        <is>
-          <t>incl. GST</t>
-        </is>
-      </c>
-      <c r="K15" s="2" t="inlineStr">
+      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>PWR LED</t>
         </is>
@@ -1283,11 +1191,11 @@
         </is>
       </c>
       <c r="B2">
-        <f>COUNTIF('Order list'!F2:F15,A2)</f>
+        <f>COUNTIF('Order list'!F2:F13,A2)</f>
         <v/>
       </c>
       <c r="C2" s="7">
-        <f>SUMIF('Order list'!F2:F15,A2,'Order list'!I2:I15)</f>
+        <f>SUMIF('Order list'!F2:F13,A2,'Order list'!I2:I13)</f>
         <v/>
       </c>
       <c r="D2" s="7">
@@ -1311,11 +1219,11 @@
         </is>
       </c>
       <c r="B3">
-        <f>COUNTIF('Order list'!F2:F15,A3)</f>
+        <f>COUNTIF('Order list'!F2:F13,A3)</f>
         <v/>
       </c>
       <c r="C3" s="7">
-        <f>SUMIF('Order list'!F2:F15,A3,'Order list'!I2:I15)</f>
+        <f>SUMIF('Order list'!F2:F13,A3,'Order list'!I2:I13)</f>
         <v/>
       </c>
       <c r="D3" s="7" t="n">
@@ -1406,7 +1314,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1623,12 +1531,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>X2 capacitor 0.1uF 275VAC</t>
+          <t>Pluggable terminal 2-pin 3.81 (5V DC in)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>C16</t>
+          <t>J5</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -1636,7 +1544,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>ECQ-UAAF104M</t>
+          <t>TBP02R1-381-02BE + plug</t>
         </is>
       </c>
       <c r="F6" t="n">
@@ -1648,154 +1556,6 @@
         <v/>
       </c>
       <c r="I6" t="inlineStr">
-        <is>
-          <t>Not found yet</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Fuse T1A 250V</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>F3</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>TR5 (Littelfuse 372)</t>
-        </is>
-      </c>
-      <c r="F7" t="n">
-        <v>6</v>
-      </c>
-      <c r="G7" s="7" t="n"/>
-      <c r="H7" s="7">
-        <f>IF(G7="","",F7*G7)</f>
-        <v/>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>Not found yet</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>NTC inrush 5R</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>RT1</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>B57236S0509M000</t>
-        </is>
-      </c>
-      <c r="F8" t="n">
-        <v>6</v>
-      </c>
-      <c r="G8" s="7" t="n">
-        <v>13.9</v>
-      </c>
-      <c r="H8" s="7">
-        <f>IF(G8="","",F8*G8)</f>
-        <v/>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>LCSC C3761585 (reference)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Terminal 2-pin 5.08mm (mains in)</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>J1</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
-        <v>1</v>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>TB007-508-02BE</t>
-        </is>
-      </c>
-      <c r="F9" t="n">
-        <v>6</v>
-      </c>
-      <c r="G9" s="7" t="n">
-        <v>48.85</v>
-      </c>
-      <c r="H9" s="7">
-        <f>IF(G9="","",F9*G9)</f>
-        <v/>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>LCSC C3816270 (reference)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Pluggable terminal 2-pin 3.81 (5V DC in)</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>J5</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
-        <v>1</v>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>TBP02R1-381-02BE + plug</t>
-        </is>
-      </c>
-      <c r="F10" t="n">
-        <v>6</v>
-      </c>
-      <c r="G10" s="7" t="n"/>
-      <c r="H10" s="7">
-        <f>IF(G10="","",F10*G10)</f>
-        <v/>
-      </c>
-      <c r="I10" t="inlineStr">
         <is>
           <t>Not found yet</t>
         </is>
@@ -1812,7 +1572,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1834,58 +1594,70 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>RS485 (isolated)</t>
+          <t>AC mains input (not used: board runs from an external 5V SMPS via J5)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>U2, U3, U4, PS2, C1, C2, C10-C15, D1-D6, F1, F2, J4, R4-R11</t>
+          <t>PS1, RV1, RT1, F3, C16, J1</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Ethernet (W5500)</t>
+          <t>RS485 (isolated)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>U7, J9, Y1, FB1, C19-C35, R20-R30</t>
+          <t>U2, U3, U4, PS2, C1, C2, C10-C15, D1-D6, F1, F2, J4, R4-R11</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Relays K1-K3</t>
+          <t>Ethernet (W5500)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>K1, K2, K3, J6, J10, J11, Q4, Q5, Q6, D9, D10, D13-D16, R13-R15, R31-R36</t>
+          <t>U7, J9, Y1, FB1, C19-C35, R20-R30</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Opto inputs</t>
+          <t>Relays K1-K3</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>U5, U6, J7, J8, JP1, JP2, D11, D12, R16-R19</t>
+          <t>K1, K2, K3, J6, J10, J11, Q4, Q5, Q6, D9, D10, D13-D16, R13-R15, R31-R36</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>Opto inputs</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>U5, U6, J7, J8, JP1, JP2, D11, D12, R16-R19</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
           <t>EEPROM</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>U8, R37, R38, C36</t>
         </is>

</xml_diff>

<commit_message>
Order list: add parts not on Sharvi/Robu (ESP32, C3, C6, C8, J5)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Order_Files/Component_Order_List.xlsx
+++ b/Order_Files/Component_Order_List.xlsx
@@ -38,7 +38,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -58,6 +58,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
     <fill>
@@ -92,7 +97,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -109,11 +114,14 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -481,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:K18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1130,6 +1138,242 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>ESP32 module</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>U1</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>ESP32-WROOM-32</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>Not on Sharvi/Robu (Balaji / other)</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="H14" s="4" t="n">
+        <v>356.19</v>
+      </c>
+      <c r="I14" s="4">
+        <f>IF(H14="","",G14*H14)</f>
+        <v/>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>LCSC reference price, not bought yet</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>LCSC C701341 (reference price)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Electrolytic 100uF 16V THT 5x11</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>C3</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>ECA-1CM101 / ECA-1CM101I</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>Not on Sharvi/Robu (Balaji / other)</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="H15" s="4" t="n"/>
+      <c r="I15" s="4">
+        <f>IF(H15="","",G15*H15)</f>
+        <v/>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>price not known yet</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>LCSC out of stock</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Tantalum 10uF 16V 3528</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>C6</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>TAJB106K016RNJ</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>Not on Sharvi/Robu (Balaji / other)</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="H16" s="4" t="n">
+        <v>18.38</v>
+      </c>
+      <c r="I16" s="4">
+        <f>IF(H16="","",G16*H16)</f>
+        <v/>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>LCSC reference price, not bought yet</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>LCSC C7193 (reference)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Capacitor 100nF 1206</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>C8</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>C1206C104K5RACTU</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>Not on Sharvi/Robu (Balaji / other)</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="H17" s="4" t="n">
+        <v>4.39</v>
+      </c>
+      <c r="I17" s="4">
+        <f>IF(H17="","",G17*H17)</f>
+        <v/>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>LCSC reference price, not bought yet</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>LCSC C41430990 (reference)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Pluggable terminal 2-pin 3.81 (5V DC in)</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>J5</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>TBP02R1-381-02BE + plug</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>Not on Sharvi/Robu (Balaji / other)</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="H18" s="4" t="n"/>
+      <c r="I18" s="4">
+        <f>IF(H18="","",G18*H18)</f>
+        <v/>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>price not known yet</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>Not found yet</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1141,7 +1385,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="70" customWidth="1" min="1" max="1"/>
@@ -1153,32 +1397,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>Website</t>
         </is>
       </c>
-      <c r="B1" s="6" t="inlineStr">
+      <c r="B1" s="7" t="inlineStr">
         <is>
           <t>Lines</t>
         </is>
       </c>
-      <c r="C1" s="6" t="inlineStr">
+      <c r="C1" s="7" t="inlineStr">
         <is>
           <t>Subtotal (Rs)</t>
         </is>
       </c>
-      <c r="D1" s="6" t="inlineStr">
+      <c r="D1" s="7" t="inlineStr">
         <is>
           <t>GST (Rs)</t>
         </is>
       </c>
-      <c r="E1" s="6" t="inlineStr">
+      <c r="E1" s="7" t="inlineStr">
         <is>
           <t>Total (Rs)</t>
         </is>
       </c>
-      <c r="F1" s="6" t="inlineStr">
+      <c r="F1" s="7" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
@@ -1191,18 +1435,18 @@
         </is>
       </c>
       <c r="B2">
-        <f>COUNTIF('Order list'!F2:F13,A2)</f>
-        <v/>
-      </c>
-      <c r="C2" s="7">
-        <f>SUMIF('Order list'!F2:F13,A2,'Order list'!I2:I13)</f>
-        <v/>
-      </c>
-      <c r="D2" s="7">
+        <f>COUNTIF('Order list'!F2:F18,A2)</f>
+        <v/>
+      </c>
+      <c r="C2" s="8">
+        <f>SUMIF('Order list'!F2:F18,A2,'Order list'!I2:I18)</f>
+        <v/>
+      </c>
+      <c r="D2" s="8">
         <f>C2*0.18</f>
         <v/>
       </c>
-      <c r="E2" s="7">
+      <c r="E2" s="8">
         <f>C2+D2</f>
         <v/>
       </c>
@@ -1219,17 +1463,17 @@
         </is>
       </c>
       <c r="B3">
-        <f>COUNTIF('Order list'!F2:F13,A3)</f>
-        <v/>
-      </c>
-      <c r="C3" s="7">
-        <f>SUMIF('Order list'!F2:F13,A3,'Order list'!I2:I13)</f>
-        <v/>
-      </c>
-      <c r="D3" s="7" t="n">
+        <f>COUNTIF('Order list'!F2:F18,A3)</f>
+        <v/>
+      </c>
+      <c r="C3" s="8">
+        <f>SUMIF('Order list'!F2:F18,A3,'Order list'!I2:I18)</f>
+        <v/>
+      </c>
+      <c r="D3" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="E3" s="7">
+      <c r="E3" s="8">
         <f>C3+D3</f>
         <v/>
       </c>
@@ -1240,61 +1484,76 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>Total (Sharvi + Robu)</t>
         </is>
       </c>
-      <c r="B4" s="8">
+      <c r="B4" s="9">
         <f>B2+B3</f>
         <v/>
       </c>
-      <c r="C4" s="9">
+      <c r="C4" s="10">
         <f>C2+C3</f>
         <v/>
       </c>
-      <c r="D4" s="9">
+      <c r="D4" s="10">
         <f>D2+D3</f>
         <v/>
       </c>
-      <c r="E4" s="9">
+      <c r="E4" s="10">
         <f>E2+E3</f>
         <v/>
       </c>
-      <c r="F4" s="8" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>JLCPCB: the same full PCB (5 pcs, 95.5 x 153.52 mm), USD 11.10 + shipping</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>In JLCPCB cart; payment pending</t>
+      <c r="F4" s="9" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Not on Sharvi/Robu (Balaji / other)</t>
+        </is>
+      </c>
+      <c r="B5">
+        <f>COUNTIF('Order list'!F2:F18,A5)</f>
+        <v/>
+      </c>
+      <c r="C5" s="8">
+        <f>SUMIF('Order list'!F2:F18,A5,'Order list'!I2:I18)</f>
+        <v/>
+      </c>
+      <c r="D5" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="8">
+        <f>C5+D5</f>
+        <v/>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Reference prices only (some unknown); not in any cart</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>This list is only for a P10-display-only build: ESP32 + P10 connector + 5V/3V3 power + programming/auto-reset + PWR LED.</t>
+          <t>JLCPCB: the same full PCB (5 pcs, 95.5 x 153.52 mm), USD 11.10 + shipping</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>In JLCPCB cart; payment pending</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>On the full PCB leave the RS485, Ethernet, relay, input and EEPROM parts unfitted (see sheet 'Not fitted (DNP)').</t>
+          <t>This list is only for a P10-display-only build: ESP32 + P10 connector + 5V/3V3 power + programming/auto-reset + PWR LED.</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
@@ -1302,6 +1561,18 @@
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>On the full PCB leave the RS485, Ethernet, relay, input and EEPROM parts unfitted (see sheet 'Not fitted (DNP)').</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1329,47 +1600,47 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="10" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Sr</t>
         </is>
       </c>
-      <c r="B1" s="10" t="inlineStr">
+      <c r="B1" s="11" t="inlineStr">
         <is>
           <t>Component</t>
         </is>
       </c>
-      <c r="C1" s="10" t="inlineStr">
+      <c r="C1" s="11" t="inlineStr">
         <is>
           <t>Designators</t>
         </is>
       </c>
-      <c r="D1" s="10" t="inlineStr">
+      <c r="D1" s="11" t="inlineStr">
         <is>
           <t>Pieces per board</t>
         </is>
       </c>
-      <c r="E1" s="10" t="inlineStr">
+      <c r="E1" s="11" t="inlineStr">
         <is>
           <t>Part number needed</t>
         </is>
       </c>
-      <c r="F1" s="10" t="inlineStr">
+      <c r="F1" s="11" t="inlineStr">
         <is>
           <t>Quantity needed (5 boards + spare)</t>
         </is>
       </c>
-      <c r="G1" s="10" t="inlineStr">
+      <c r="G1" s="11" t="inlineStr">
         <is>
           <t>Reference price per piece (Rs, LCSC)</t>
         </is>
       </c>
-      <c r="H1" s="10" t="inlineStr">
+      <c r="H1" s="11" t="inlineStr">
         <is>
           <t>Reference total (Rs)</t>
         </is>
       </c>
-      <c r="I1" s="10" t="inlineStr">
+      <c r="I1" s="11" t="inlineStr">
         <is>
           <t>Status / note</t>
         </is>
@@ -1400,10 +1671,10 @@
       <c r="F2" t="n">
         <v>6</v>
       </c>
-      <c r="G2" s="7" t="n">
+      <c r="G2" s="8" t="n">
         <v>356.19</v>
       </c>
-      <c r="H2" s="7">
+      <c r="H2" s="8">
         <f>IF(G2="","",F2*G2)</f>
         <v/>
       </c>
@@ -1438,8 +1709,8 @@
       <c r="F3" t="n">
         <v>6</v>
       </c>
-      <c r="G3" s="7" t="n"/>
-      <c r="H3" s="7">
+      <c r="G3" s="8" t="n"/>
+      <c r="H3" s="8">
         <f>IF(G3="","",F3*G3)</f>
         <v/>
       </c>
@@ -1474,10 +1745,10 @@
       <c r="F4" t="n">
         <v>6</v>
       </c>
-      <c r="G4" s="7" t="n">
+      <c r="G4" s="8" t="n">
         <v>18.38</v>
       </c>
-      <c r="H4" s="7">
+      <c r="H4" s="8">
         <f>IF(G4="","",F4*G4)</f>
         <v/>
       </c>
@@ -1512,10 +1783,10 @@
       <c r="F5" t="n">
         <v>6</v>
       </c>
-      <c r="G5" s="7" t="n">
+      <c r="G5" s="8" t="n">
         <v>4.39</v>
       </c>
-      <c r="H5" s="7">
+      <c r="H5" s="8">
         <f>IF(G5="","",F5*G5)</f>
         <v/>
       </c>
@@ -1550,8 +1821,8 @@
       <c r="F6" t="n">
         <v>6</v>
       </c>
-      <c r="G6" s="7" t="n"/>
-      <c r="H6" s="7">
+      <c r="G6" s="8" t="n"/>
+      <c r="H6" s="8">
         <f>IF(G6="","",F6*G6)</f>
         <v/>
       </c>
@@ -1580,12 +1851,12 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>Circuit</t>
         </is>
       </c>
-      <c r="B1" s="6" t="inlineStr">
+      <c r="B1" s="7" t="inlineStr">
         <is>
           <t>Designators left unfitted</t>
         </is>

</xml_diff>